<commit_message>
Integration und Interpolation umgesetzt
</commit_message>
<xml_diff>
--- a/Zeitplan.xlsx
+++ b/Zeitplan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benne\OneDrive\Desktop\Taschenrechner_Vendl\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benne\OneDrive\Desktop\6.Semester\Numerischer_Taschenrechner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71440965-7B84-4FD8-88DF-FE8138CD7ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3243918-F0BF-4F54-86BF-C78431E7C6D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Startdatum</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t xml:space="preserve">ggf. Verbesserungen vom Kunden; Puffer; ggf. Verbesserung vom GUI; ggf. Umsetzung von Zusatzfunktionen wie Basistaschenrechner </t>
+  </si>
+  <si>
+    <t>Newton Cotes verbessern bezüglich Doppelstreifen</t>
   </si>
 </sst>
 </file>
@@ -574,7 +577,7 @@
     <col min="2" max="2" width="25.6328125" customWidth="1"/>
     <col min="3" max="3" width="24.1796875" customWidth="1"/>
     <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="5" width="21.90625" customWidth="1"/>
+    <col min="5" max="5" width="57.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
@@ -620,9 +623,11 @@
         <v>46108</v>
       </c>
       <c r="D4" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">

</xml_diff>